<commit_message>
Updating data dictionary, beginning cleaning process
</commit_message>
<xml_diff>
--- a/DataDictionary.xlsx
+++ b/DataDictionary.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsleylotito/Library/CloudStorage/Dropbox-InsightExposure/Ainsley Lotito/Silica_OSHA_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A0B31C1-0A0C-DE41-8638-633A88BED3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBCD6E34-9C17-3F4F-B24F-46E5BC6F736D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1400" windowWidth="27640" windowHeight="16680" xr2:uid="{0EEC19A2-9898-F84A-B445-76508146080C}"/>
+    <workbookView xWindow="1500" yWindow="1400" windowWidth="27640" windowHeight="16680" activeTab="1" xr2:uid="{0EEC19A2-9898-F84A-B445-76508146080C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Intro" sheetId="3" r:id="rId1"/>
+    <sheet name="OSHA Raw Data Dictionary" sheetId="1" r:id="rId2"/>
+    <sheet name="Cleaned Dataset Dictionary" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,11 +40,244 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
+  <si>
+    <r>
+      <t xml:space="preserve">To view all variables imported from the raw OSHA datafile, navigate to the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>OSHA Raw Data Dictionary sheet.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>To view all variables retained for the Cleaned analytic dataset, including a description of newly created variables, navigate to the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Cleaned Dataset Dictionary Sheet.</t>
+    </r>
+  </si>
+  <si>
+    <t>Variable Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Levels/Values</t>
+  </si>
+  <si>
+    <t>INSPECTION</t>
+  </si>
+  <si>
+    <t>SAMPLING_NUMBER</t>
+  </si>
+  <si>
+    <t>OFFICE</t>
+  </si>
+  <si>
+    <t>ESTABLISHMENT</t>
+  </si>
+  <si>
+    <t>SIC</t>
+  </si>
+  <si>
+    <t>NAICS</t>
+  </si>
+  <si>
+    <t>CSHO</t>
+  </si>
+  <si>
+    <t>DATE_SAMPLED</t>
+  </si>
+  <si>
+    <t>DATE_REPORTED</t>
+  </si>
+  <si>
+    <t>EIGHTHR</t>
+  </si>
+  <si>
+    <t>INSTRUMENT</t>
+  </si>
+  <si>
+    <t>LAB_NUMBER</t>
+  </si>
+  <si>
+    <t>FIELD_NUMBER</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>BLANK</t>
+  </si>
+  <si>
+    <t>TIME</t>
+  </si>
+  <si>
+    <t>AIR_VOLUME</t>
+  </si>
+  <si>
+    <t>WEIGHT</t>
+  </si>
+  <si>
+    <t>IMIS</t>
+  </si>
+  <si>
+    <t>SUBSTANCE</t>
+  </si>
+  <si>
+    <t>RESULT</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
+    <t>QUALIFIER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Dictionary: https://www.osha.gov/opengov/osha-health-samples-dataset-field-definitions </t>
+  </si>
+  <si>
+    <t>Establishment Name</t>
+  </si>
+  <si>
+    <t>Unique identifier tied to individual sample media submitted for analysis</t>
+  </si>
+  <si>
+    <t>Laboratory instrument type used for analysis</t>
+  </si>
+  <si>
+    <t>Sample type</t>
+  </si>
+  <si>
+    <t>P - Personal, A - Area, B - Bulk, W - Wipe</t>
+  </si>
+  <si>
+    <t>Sample represents a blank used for analysis</t>
+  </si>
+  <si>
+    <t>Y,N</t>
+  </si>
+  <si>
+    <t>Time sampled in minutes</t>
+  </si>
+  <si>
+    <t>Air volume sampled in liters</t>
+  </si>
+  <si>
+    <t>Sample weight for bulks and silica samples</t>
+  </si>
+  <si>
+    <t>IMIS Substance code number assigned by OSHA to each substance</t>
+  </si>
+  <si>
+    <t>Chemical Name</t>
+  </si>
+  <si>
+    <t>Sample result from laboratory analysis for each sample submitted with a unique field number</t>
+  </si>
+  <si>
+    <t>Unit of measurement from IMIS manual.</t>
+  </si>
+  <si>
+    <t>M - mg/m3, X - micrograms, P - parts per million, Y - milligrams, F - fibers/cc, % - percentage</t>
+  </si>
+  <si>
+    <t>Result qualifier values</t>
+  </si>
+  <si>
+    <t>ND - result less than quantification limit, BLK - Blank, @ - Approximately, etc.</t>
+  </si>
+  <si>
+    <t>Unique identifier tied to inspection- nine numbers in length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicates the 4-digit Standard Industrial Classification Code from the 1987 version SIC manual which most closely applies. </t>
+  </si>
+  <si>
+    <t>North American Industrial Classification Code System Code</t>
+  </si>
+  <si>
+    <t>Unique identifier tied to single exposure assessment. There may be multiple media tied to this number, reflecting multiple samples in a time-weighted sample</t>
+  </si>
+  <si>
+    <t>Unique number assigned to an OSHA office</t>
+  </si>
+  <si>
+    <t>Date the sample was taken</t>
+  </si>
+  <si>
+    <t>Date the results were released to the OSHA office</t>
+  </si>
+  <si>
+    <t>Eight hour TWA calculation used</t>
+  </si>
+  <si>
+    <t>Unique identifier assigned by laboratory for internal use</t>
+  </si>
+  <si>
+    <t>5 digits followed by a letter</t>
+  </si>
+  <si>
+    <t>Not in dictionary, possibly pertains to whether inspection was conducted by a Compliance Safety Health Officer</t>
+  </si>
+  <si>
+    <t>Y/N</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -57,7 +292,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -65,17 +300,175 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -86,6 +479,18 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{16C53CA2-5A24-4540-B934-424157BF101C}" name="Table1" displayName="Table1" ref="A1:C24" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4" headerRowBorderDxfId="5" tableBorderDxfId="6">
+  <autoFilter ref="A1:C24" xr:uid="{16C53CA2-5A24-4540-B934-424157BF101C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{6725AEAF-D16C-4347-B168-F0B7E7DB5D00}" name="Variable Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{8781854F-FD77-2A41-A2A9-09CC4A7D59DA}" name="Description" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{614E54A8-5D6B-0440-9C28-048CE3156CA0}" name="Levels/Values" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -404,7 +809,285 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DEA2A6B-AC72-B44C-B2CE-50A91214F662}">
+  <dimension ref="A2:A6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="141" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" ht="27" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="56" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C1DD773-568A-BC4E-B6FC-43C06C044029}">
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33.5" customWidth="1"/>
+    <col min="2" max="2" width="90.5" style="8" customWidth="1"/>
+    <col min="3" max="3" width="27.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" spans="1:3" ht="69" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="6"/>
+    </row>
+    <row r="4" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6"/>
+    </row>
+    <row r="5" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" ht="46" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="6"/>
+    </row>
+    <row r="7" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" ht="46" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" ht="46" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="6"/>
+    </row>
+    <row r="15" spans="1:3" ht="46" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" ht="23" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="6"/>
+    </row>
+    <row r="22" spans="1:3" ht="46" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" ht="138" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="92" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DB83832-47BE-EE4F-A03F-1A398FA8A7BF}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>

</xml_diff>